<commit_message>
Update master_template_rab.xlsx from local laptop
</commit_message>
<xml_diff>
--- a/public/templates/master_template_rab.xlsx
+++ b/public/templates/master_template_rab.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\data\Aplikasi\Zona Geometry-App\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADD2823-90FE-4CB8-8BD1-61B505EE4EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB89A878-21B0-4EDD-87E2-D8BBF85F7BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{5E860003-9DCC-49E7-B9D8-7C8CA0B8260C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5E860003-9DCC-49E7-B9D8-7C8CA0B8260C}"/>
   </bookViews>
   <sheets>
     <sheet name="harga_satuan_terpakai" sheetId="8" r:id="rId1"/>
@@ -693,7 +693,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="19">
     <dxf>
       <fill>
         <patternFill>
@@ -718,6 +718,73 @@
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -10842,10 +10909,10 @@
     <mergeCell ref="C5:D5"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="12" priority="1">
+    <cfRule type="expression" dxfId="18" priority="1">
       <formula>$K6=",..,"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="2">
+    <cfRule type="expression" dxfId="17" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -34977,20 +35044,20 @@
     <mergeCell ref="B4:H4"/>
   </mergeCells>
   <conditionalFormatting sqref="B7:B996 E7:H996">
-    <cfRule type="expression" dxfId="10" priority="6">
+    <cfRule type="expression" dxfId="16" priority="6">
       <formula>$J7=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:H996">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="15" priority="1">
       <formula>AND(LEN($B7)=1,$C7&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>$C7&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7:D996">
-    <cfRule type="expression" dxfId="7" priority="8">
+    <cfRule type="expression" dxfId="13" priority="8">
       <formula>$J7=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -37307,29 +37374,26 @@
     <mergeCell ref="C6:D6"/>
   </mergeCells>
   <conditionalFormatting sqref="B8:N16999">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="12" priority="1">
       <formula>$P7=",..,"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="11" priority="2">
       <formula>AND(LEN($B8)=1,$C8&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="10" priority="3">
       <formula>$C8&lt;&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="9" priority="4">
       <formula>AND(LEN($B8)&lt;&gt;0,$D8&lt;&gt;0)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5">
-      <formula>AND($D8&lt;&gt;0,$G8=0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8:H16999">
-    <cfRule type="expression" dxfId="1" priority="7">
+    <cfRule type="expression" dxfId="8" priority="7">
       <formula>IF(G8&lt;&gt;"", NOT(AND(OR(LEFT($E8,2)="L.", LEFT($E8,2)="A.", LEFT($E8,2)="B.", LEFT($E8,2)="M."), $H8&lt;&gt;"", $E8&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8:K16999">
-    <cfRule type="notContainsBlanks" dxfId="0" priority="6">
+    <cfRule type="notContainsBlanks" dxfId="7" priority="6">
       <formula>LEN(TRIM(H8))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Final template update: master_template_rab.xlsx
</commit_message>
<xml_diff>
--- a/public/templates/master_template_rab.xlsx
+++ b/public/templates/master_template_rab.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9057A17D-1A69-4EBF-9DBF-0DABE0F4E1FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82D3C60-F672-496C-ABD6-7110C327D5E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="harga satuan terpakai" sheetId="8" r:id="rId1"/>
@@ -19,7 +19,20 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">ahsp!$1:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">hsp!$1:$6</definedName>
   </definedNames>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -435,7 +448,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="15">
     <dxf>
       <fill>
         <patternFill>
@@ -481,6 +494,65 @@
       <fill>
         <patternFill>
           <bgColor theme="7" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <color rgb="FFFFC000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -9434,7 +9506,7 @@
     <mergeCell ref="C5:D5"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:I2685">
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>AND($C6&lt;&gt;0,$G6=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11670,23 +11742,26 @@
     <mergeCell ref="C6:D6"/>
   </mergeCells>
   <conditionalFormatting sqref="B7:N16998">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="8" priority="1">
       <formula>AND(LEN($B7)=1,$C7&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="7" priority="3">
       <formula>$C7&lt;&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>AND(LEN($B7)&lt;&gt;0,$D7&lt;&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="4">
+      <formula>AND(LEN($B7)=1,$D7&lt;&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:H16998">
-    <cfRule type="expression" dxfId="1" priority="7">
+    <cfRule type="expression" dxfId="10" priority="8">
       <formula>IF(G7&lt;&gt;"", NOT(AND(OR(LEFT($E7,2)="L.", LEFT($E7,2)="A.", LEFT($E7,2)="B.", LEFT($E7,2)="M."), $H7&lt;&gt;"", $E7&lt;&gt;"")),FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:K16998">
-    <cfRule type="notContainsBlanks" dxfId="0" priority="6">
+    <cfRule type="notContainsBlanks" dxfId="9" priority="7">
       <formula>LEN(TRIM(H7))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -35785,15 +35860,15 @@
     <mergeCell ref="B4:H4"/>
   </mergeCells>
   <conditionalFormatting sqref="B7:B996 E7:H996">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="13" priority="6">
       <formula>$J7=",..,"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:H996">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="12" priority="1">
       <formula>AND(LEN($B7)=1,$C7&lt;&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="11" priority="2">
       <formula>$C7&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>